<commit_message>
[유민형][System] Ability PrefabPath 작성
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Ability.xlsx
+++ b/JsonConverter/ExcelFiles/Ability.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OZ_Project\Fantastic4\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F6EB691-0C3B-4FC6-A15F-8EE924E8ADEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49E04AC3-1D30-4C02-80DB-41EE7EB6E8EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
   <si>
     <t>Ability 고유 ID</t>
   </si>
@@ -101,6 +101,10 @@
   </si>
   <si>
     <t>Prefab/Ability/HealField</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>PrefabPath</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -553,7 +557,9 @@
       <c r="E3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="5"/>
+      <c r="F3" s="5" t="s">
+        <v>23</v>
+      </c>
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>

</xml_diff>